<commit_message>
Update data - 2026-09-19 18:49:36
</commit_message>
<xml_diff>
--- a/l9.xlsx
+++ b/l9.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Spare_Parts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Preventive_Maintenance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Spare_Parts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Preventive_Maintenance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="store" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,52 +416,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Part_Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tension</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Available_Quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Lead_Time</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Is_Critical</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Image_URL</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -470,6 +429,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Part_Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Available_Quantity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Lead_Time</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Is_Critical</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -523,4 +538,75 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Repair_Duration</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Event_Fault</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Corrective_Action</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Performed_By</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Spare_Parts_Used</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Fault_Type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Technician_Skill</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Safety_Compliance</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update data - 2026-09-19 18:50:23
</commit_message>
<xml_diff>
--- a/l9.xlsx
+++ b/l9.xlsx
@@ -7,10 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Spare_Parts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Preventive_Maintenance" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="store" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Spare_Parts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Preventive_Maintenance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="store" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,9 +415,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Part_Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Available_Quantity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Lead_Time</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Is_Critical</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -429,46 +471,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Part_Name</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Maintenance_Type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Tension</t>
+          <t>Task_Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Available_Quantity</t>
+          <t>Period_Days</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Lead_Time</t>
+          <t>Last_Execution</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Is_Critical</t>
+          <t>Next_Date</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
+        <is>
+          <t>Default_Spare_Part</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>Image_URL</t>
         </is>
@@ -485,67 +532,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Maintenance_Type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Task_Name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Period_Days</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Last_Execution</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Next_Date</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Default_Spare_Part</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Image_URL</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Update data - 2026-09-19 18:52:33
</commit_message>
<xml_diff>
--- a/l9.xlsx
+++ b/l9.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Spare_Parts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Preventive_Maintenance" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="store" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Electric" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -595,4 +596,75 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Repair_Duration</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Event_Fault</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Corrective_Action</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Performed_By</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Spare_Parts_Used</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Fault_Type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Technician_Skill</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Safety_Compliance</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>